<commit_message>
Updated EDA summary code and excel summary files
</commit_message>
<xml_diff>
--- a/outputs/EDA_transaction_with_graph_features_Old.xlsx
+++ b/outputs/EDA_transaction_with_graph_features_Old.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/fc4bd521ffc22738/Desktop/Freelancing/AIGEN/smartsentry_aml_model/outputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="13_ncr:1_{E7AB24AF-35A9-0742-9CE2-464F1FC838D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0899F591-F7E6-44A1-A2A8-6071DFE3CDDD}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="13_ncr:1_{E7AB24AF-35A9-0742-9CE2-464F1FC838D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BC879C5E-8F00-43DB-8A67-2B16F8B6CE24}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1_Overview" sheetId="1" r:id="rId1"/>
@@ -3278,7 +3278,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -3396,10 +3396,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -3432,6 +3428,19 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3739,8 +3748,8 @@
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
-    <col min="2" max="2" width="25" customWidth="1"/>
-    <col min="3" max="4" width="20" customWidth="1"/>
+    <col min="2" max="2" width="25" style="51" customWidth="1"/>
+    <col min="3" max="4" width="20" style="51" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="21" x14ac:dyDescent="0.3">
@@ -3760,7 +3769,7 @@
       <c r="A4" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="54" t="s">
         <v>4</v>
       </c>
     </row>
@@ -3768,7 +3777,7 @@
       <c r="A5" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="55" t="s">
         <v>6</v>
       </c>
     </row>
@@ -3776,7 +3785,7 @@
       <c r="A6" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="54" t="s">
         <v>8</v>
       </c>
     </row>
@@ -3784,7 +3793,7 @@
       <c r="A7" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="55" t="s">
         <v>10</v>
       </c>
     </row>
@@ -3792,7 +3801,7 @@
       <c r="A8" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="54" t="s">
         <v>12</v>
       </c>
     </row>
@@ -3800,7 +3809,7 @@
       <c r="A9" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="55" t="s">
         <v>14</v>
       </c>
     </row>
@@ -3808,7 +3817,7 @@
       <c r="A10" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="54" t="s">
         <v>16</v>
       </c>
     </row>
@@ -3816,7 +3825,7 @@
       <c r="A11" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="55" t="s">
         <v>18</v>
       </c>
     </row>
@@ -3824,7 +3833,7 @@
       <c r="A12" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="54" t="s">
         <v>20</v>
       </c>
     </row>
@@ -3832,7 +3841,7 @@
       <c r="A13" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="B13" s="55" t="s">
         <v>22</v>
       </c>
     </row>
@@ -3840,7 +3849,7 @@
       <c r="A14" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="54" t="s">
         <v>24</v>
       </c>
     </row>
@@ -3848,7 +3857,7 @@
       <c r="A15" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="B15" s="55" t="s">
         <v>26</v>
       </c>
     </row>
@@ -3856,7 +3865,7 @@
       <c r="A16" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="54" t="s">
         <v>28</v>
       </c>
     </row>
@@ -3864,7 +3873,7 @@
       <c r="A17" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B17" s="6" t="s">
+      <c r="B17" s="55" t="s">
         <v>30</v>
       </c>
     </row>
@@ -3891,13 +3900,13 @@
       <c r="A22" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="B22" s="6">
+      <c r="B22" s="55">
         <v>75083</v>
       </c>
-      <c r="C22" s="6" t="s">
+      <c r="C22" s="55" t="s">
         <v>37</v>
       </c>
-      <c r="D22" s="6" t="s">
+      <c r="D22" s="55" t="s">
         <v>38</v>
       </c>
     </row>
@@ -3905,13 +3914,13 @@
       <c r="A23" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="B23" s="9">
+      <c r="B23" s="56">
         <v>4800</v>
       </c>
-      <c r="C23" s="9" t="s">
+      <c r="C23" s="56" t="s">
         <v>40</v>
       </c>
-      <c r="D23" s="9" t="s">
+      <c r="D23" s="56" t="s">
         <v>41</v>
       </c>
     </row>
@@ -3919,13 +3928,13 @@
       <c r="A24" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="B24" s="9">
+      <c r="B24" s="56">
         <v>2706</v>
       </c>
-      <c r="C24" s="9" t="s">
+      <c r="C24" s="56" t="s">
         <v>43</v>
       </c>
-      <c r="D24" s="9" t="s">
+      <c r="D24" s="56" t="s">
         <v>41</v>
       </c>
     </row>
@@ -3933,13 +3942,13 @@
       <c r="A25" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="B25" s="9">
+      <c r="B25" s="56">
         <v>2387</v>
       </c>
-      <c r="C25" s="9" t="s">
+      <c r="C25" s="56" t="s">
         <v>45</v>
       </c>
-      <c r="D25" s="9" t="s">
+      <c r="D25" s="56" t="s">
         <v>41</v>
       </c>
     </row>
@@ -3947,13 +3956,13 @@
       <c r="A26" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="B26" s="9">
+      <c r="B26" s="56">
         <v>2000</v>
       </c>
-      <c r="C26" s="9" t="s">
+      <c r="C26" s="56" t="s">
         <v>47</v>
       </c>
-      <c r="D26" s="9" t="s">
+      <c r="D26" s="56" t="s">
         <v>41</v>
       </c>
     </row>
@@ -3961,13 +3970,13 @@
       <c r="A27" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="B27" s="9">
+      <c r="B27" s="56">
         <v>22</v>
       </c>
-      <c r="C27" s="9" t="s">
+      <c r="C27" s="56" t="s">
         <v>49</v>
       </c>
-      <c r="D27" s="9" t="s">
+      <c r="D27" s="56" t="s">
         <v>41</v>
       </c>
     </row>
@@ -3994,13 +4003,13 @@
       <c r="A32" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="B32" s="4">
+      <c r="B32" s="54">
         <v>8778</v>
       </c>
-      <c r="C32" s="4">
+      <c r="C32" s="54">
         <v>1184</v>
       </c>
-      <c r="D32" s="4" t="s">
+      <c r="D32" s="54" t="s">
         <v>56</v>
       </c>
     </row>
@@ -4008,13 +4017,13 @@
       <c r="A33" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="B33" s="6">
+      <c r="B33" s="55">
         <v>8575</v>
       </c>
-      <c r="C33" s="6">
+      <c r="C33" s="55">
         <v>1203</v>
       </c>
-      <c r="D33" s="6" t="s">
+      <c r="D33" s="55" t="s">
         <v>58</v>
       </c>
     </row>
@@ -4022,13 +4031,13 @@
       <c r="A34" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="B34" s="4">
+      <c r="B34" s="54">
         <v>42073</v>
       </c>
-      <c r="C34" s="4">
+      <c r="C34" s="54">
         <v>4759</v>
       </c>
-      <c r="D34" s="4" t="s">
+      <c r="D34" s="54" t="s">
         <v>60</v>
       </c>
     </row>
@@ -4036,13 +4045,13 @@
       <c r="A35" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="B35" s="6">
+      <c r="B35" s="55">
         <v>27572</v>
       </c>
-      <c r="C35" s="6">
+      <c r="C35" s="55">
         <v>4769</v>
       </c>
-      <c r="D35" s="6" t="s">
+      <c r="D35" s="55" t="s">
         <v>62</v>
       </c>
     </row>
@@ -4077,14 +4086,14 @@
       <c r="F3" s="37"/>
     </row>
     <row r="4" spans="1:6" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="41" t="s">
+      <c r="A4" s="52" t="s">
         <v>920</v>
       </c>
-      <c r="B4" s="42"/>
-      <c r="C4" s="42"/>
-      <c r="D4" s="42"/>
-      <c r="E4" s="42"/>
-      <c r="F4" s="42"/>
+      <c r="B4" s="53"/>
+      <c r="C4" s="53"/>
+      <c r="D4" s="53"/>
+      <c r="E4" s="53"/>
+      <c r="F4" s="53"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="8" t="s">
@@ -4309,14 +4318,14 @@
       <c r="F24" s="37"/>
     </row>
     <row r="25" spans="1:6" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="41" t="s">
+      <c r="A25" s="52" t="s">
         <v>957</v>
       </c>
-      <c r="B25" s="42"/>
-      <c r="C25" s="42"/>
-      <c r="D25" s="42"/>
-      <c r="E25" s="42"/>
-      <c r="F25" s="42"/>
+      <c r="B25" s="53"/>
+      <c r="C25" s="53"/>
+      <c r="D25" s="53"/>
+      <c r="E25" s="53"/>
+      <c r="F25" s="53"/>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="8" t="s">
@@ -4541,14 +4550,14 @@
       <c r="F45" s="37"/>
     </row>
     <row r="46" spans="1:6" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="41" t="s">
+      <c r="A46" s="52" t="s">
         <v>969</v>
       </c>
-      <c r="B46" s="42"/>
-      <c r="C46" s="42"/>
-      <c r="D46" s="42"/>
-      <c r="E46" s="42"/>
-      <c r="F46" s="42"/>
+      <c r="B46" s="53"/>
+      <c r="C46" s="53"/>
+      <c r="D46" s="53"/>
+      <c r="E46" s="53"/>
+      <c r="F46" s="53"/>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A47" s="8" t="s">
@@ -4773,14 +4782,14 @@
       <c r="F66" s="37"/>
     </row>
     <row r="67" spans="1:6" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A67" s="41" t="s">
+      <c r="A67" s="52" t="s">
         <v>980</v>
       </c>
-      <c r="B67" s="42"/>
-      <c r="C67" s="42"/>
-      <c r="D67" s="42"/>
-      <c r="E67" s="42"/>
-      <c r="F67" s="42"/>
+      <c r="B67" s="53"/>
+      <c r="C67" s="53"/>
+      <c r="D67" s="53"/>
+      <c r="E67" s="53"/>
+      <c r="F67" s="53"/>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A68" s="8" t="s">
@@ -5005,14 +5014,14 @@
       <c r="F87" s="37"/>
     </row>
     <row r="88" spans="1:6" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A88" s="41" t="s">
+      <c r="A88" s="52" t="s">
         <v>995</v>
       </c>
-      <c r="B88" s="42"/>
-      <c r="C88" s="42"/>
-      <c r="D88" s="42"/>
-      <c r="E88" s="42"/>
-      <c r="F88" s="42"/>
+      <c r="B88" s="53"/>
+      <c r="C88" s="53"/>
+      <c r="D88" s="53"/>
+      <c r="E88" s="53"/>
+      <c r="F88" s="53"/>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A89" s="8" t="s">
@@ -7618,7 +7627,7 @@
   <dimension ref="A1:E131"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="31.33203125" style="53" customWidth="1"/>
+    <col min="1" max="1" width="31.33203125" style="51" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
     <col min="3" max="3" width="22" customWidth="1"/>
     <col min="4" max="4" width="60" customWidth="1"/>
@@ -7648,7 +7657,7 @@
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" s="43" t="s">
+      <c r="A3" s="41" t="s">
         <v>69</v>
       </c>
       <c r="B3" s="12" t="s">
@@ -7665,7 +7674,7 @@
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A4" s="43" t="s">
+      <c r="A4" s="41" t="s">
         <v>74</v>
       </c>
       <c r="B4" s="12" t="s">
@@ -7682,7 +7691,7 @@
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5" s="43" t="s">
+      <c r="A5" s="41" t="s">
         <v>77</v>
       </c>
       <c r="B5" s="12" t="s">
@@ -7699,7 +7708,7 @@
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A6" s="43" t="s">
+      <c r="A6" s="41" t="s">
         <v>79</v>
       </c>
       <c r="B6" s="12" t="s">
@@ -7716,7 +7725,7 @@
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A7" s="43" t="s">
+      <c r="A7" s="41" t="s">
         <v>81</v>
       </c>
       <c r="B7" s="12" t="s">
@@ -7733,7 +7742,7 @@
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8" s="43" t="s">
+      <c r="A8" s="41" t="s">
         <v>83</v>
       </c>
       <c r="B8" s="12" t="s">
@@ -7750,7 +7759,7 @@
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A9" s="43" t="s">
+      <c r="A9" s="41" t="s">
         <v>85</v>
       </c>
       <c r="B9" s="12" t="s">
@@ -7767,7 +7776,7 @@
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10" s="43" t="s">
+      <c r="A10" s="41" t="s">
         <v>87</v>
       </c>
       <c r="B10" s="12" t="s">
@@ -7784,7 +7793,7 @@
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A11" s="43" t="s">
+      <c r="A11" s="41" t="s">
         <v>90</v>
       </c>
       <c r="B11" s="12" t="s">
@@ -7801,7 +7810,7 @@
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A12" s="43" t="s">
+      <c r="A12" s="41" t="s">
         <v>93</v>
       </c>
       <c r="B12" s="12" t="s">
@@ -7818,7 +7827,7 @@
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A13" s="43" t="s">
+      <c r="A13" s="41" t="s">
         <v>95</v>
       </c>
       <c r="B13" s="12" t="s">
@@ -7835,7 +7844,7 @@
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A14" s="43" t="s">
+      <c r="A14" s="41" t="s">
         <v>97</v>
       </c>
       <c r="B14" s="12" t="s">
@@ -7852,7 +7861,7 @@
       </c>
     </row>
     <row r="15" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A15" s="44" t="s">
+      <c r="A15" s="42" t="s">
         <v>101</v>
       </c>
       <c r="B15" s="14" t="s">
@@ -7869,7 +7878,7 @@
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A16" s="44" t="s">
+      <c r="A16" s="42" t="s">
         <v>105</v>
       </c>
       <c r="B16" s="14" t="s">
@@ -7886,7 +7895,7 @@
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A17" s="45" t="s">
+      <c r="A17" s="43" t="s">
         <v>108</v>
       </c>
       <c r="B17" s="16" t="s">
@@ -7903,7 +7912,7 @@
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A18" s="45" t="s">
+      <c r="A18" s="43" t="s">
         <v>111</v>
       </c>
       <c r="B18" s="16" t="s">
@@ -7920,7 +7929,7 @@
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A19" s="45" t="s">
+      <c r="A19" s="43" t="s">
         <v>114</v>
       </c>
       <c r="B19" s="16" t="s">
@@ -7937,7 +7946,7 @@
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A20" s="45" t="s">
+      <c r="A20" s="43" t="s">
         <v>116</v>
       </c>
       <c r="B20" s="16" t="s">
@@ -7954,7 +7963,7 @@
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A21" s="45" t="s">
+      <c r="A21" s="43" t="s">
         <v>118</v>
       </c>
       <c r="B21" s="16" t="s">
@@ -7971,7 +7980,7 @@
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A22" s="45" t="s">
+      <c r="A22" s="43" t="s">
         <v>120</v>
       </c>
       <c r="B22" s="16" t="s">
@@ -7988,7 +7997,7 @@
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A23" s="45" t="s">
+      <c r="A23" s="43" t="s">
         <v>122</v>
       </c>
       <c r="B23" s="16" t="s">
@@ -8005,7 +8014,7 @@
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A24" s="45" t="s">
+      <c r="A24" s="43" t="s">
         <v>124</v>
       </c>
       <c r="B24" s="16" t="s">
@@ -8022,7 +8031,7 @@
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A25" s="45" t="s">
+      <c r="A25" s="43" t="s">
         <v>126</v>
       </c>
       <c r="B25" s="16" t="s">
@@ -8039,7 +8048,7 @@
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A26" s="45" t="s">
+      <c r="A26" s="43" t="s">
         <v>128</v>
       </c>
       <c r="B26" s="16" t="s">
@@ -8056,7 +8065,7 @@
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A27" s="46" t="s">
+      <c r="A27" s="44" t="s">
         <v>130</v>
       </c>
       <c r="B27" s="18" t="s">
@@ -8073,7 +8082,7 @@
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A28" s="46" t="s">
+      <c r="A28" s="44" t="s">
         <v>133</v>
       </c>
       <c r="B28" s="18" t="s">
@@ -8090,7 +8099,7 @@
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A29" s="46" t="s">
+      <c r="A29" s="44" t="s">
         <v>135</v>
       </c>
       <c r="B29" s="18" t="s">
@@ -8107,7 +8116,7 @@
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A30" s="46" t="s">
+      <c r="A30" s="44" t="s">
         <v>137</v>
       </c>
       <c r="B30" s="18" t="s">
@@ -8124,7 +8133,7 @@
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A31" s="46" t="s">
+      <c r="A31" s="44" t="s">
         <v>139</v>
       </c>
       <c r="B31" s="18" t="s">
@@ -8141,7 +8150,7 @@
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A32" s="47" t="s">
+      <c r="A32" s="45" t="s">
         <v>141</v>
       </c>
       <c r="B32" s="19" t="s">
@@ -8158,7 +8167,7 @@
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A33" s="47" t="s">
+      <c r="A33" s="45" t="s">
         <v>144</v>
       </c>
       <c r="B33" s="19" t="s">
@@ -8175,7 +8184,7 @@
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A34" s="48" t="s">
+      <c r="A34" s="46" t="s">
         <v>146</v>
       </c>
       <c r="B34" s="21" t="s">
@@ -8192,7 +8201,7 @@
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A35" s="48" t="s">
+      <c r="A35" s="46" t="s">
         <v>150</v>
       </c>
       <c r="B35" s="21" t="s">
@@ -8209,7 +8218,7 @@
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A36" s="48" t="s">
+      <c r="A36" s="46" t="s">
         <v>153</v>
       </c>
       <c r="B36" s="21" t="s">
@@ -8226,7 +8235,7 @@
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A37" s="48" t="s">
+      <c r="A37" s="46" t="s">
         <v>156</v>
       </c>
       <c r="B37" s="21" t="s">
@@ -8243,7 +8252,7 @@
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A38" s="48" t="s">
+      <c r="A38" s="46" t="s">
         <v>159</v>
       </c>
       <c r="B38" s="21" t="s">
@@ -8260,7 +8269,7 @@
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A39" s="48" t="s">
+      <c r="A39" s="46" t="s">
         <v>162</v>
       </c>
       <c r="B39" s="21" t="s">
@@ -8277,7 +8286,7 @@
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A40" s="48" t="s">
+      <c r="A40" s="46" t="s">
         <v>165</v>
       </c>
       <c r="B40" s="21" t="s">
@@ -8294,7 +8303,7 @@
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A41" s="48" t="s">
+      <c r="A41" s="46" t="s">
         <v>168</v>
       </c>
       <c r="B41" s="21" t="s">
@@ -8311,7 +8320,7 @@
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A42" s="49" t="s">
+      <c r="A42" s="47" t="s">
         <v>171</v>
       </c>
       <c r="B42" s="23" t="s">
@@ -8328,7 +8337,7 @@
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A43" s="49" t="s">
+      <c r="A43" s="47" t="s">
         <v>175</v>
       </c>
       <c r="B43" s="23" t="s">
@@ -8345,7 +8354,7 @@
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A44" s="49" t="s">
+      <c r="A44" s="47" t="s">
         <v>178</v>
       </c>
       <c r="B44" s="23" t="s">
@@ -8362,7 +8371,7 @@
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A45" s="47" t="s">
+      <c r="A45" s="45" t="s">
         <v>181</v>
       </c>
       <c r="B45" s="19" t="s">
@@ -8379,7 +8388,7 @@
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A46" s="45" t="s">
+      <c r="A46" s="43" t="s">
         <v>184</v>
       </c>
       <c r="B46" s="16" t="s">
@@ -8396,7 +8405,7 @@
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A47" s="50" t="s">
+      <c r="A47" s="48" t="s">
         <v>187</v>
       </c>
       <c r="B47" s="25" t="s">
@@ -8413,7 +8422,7 @@
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A48" s="50" t="s">
+      <c r="A48" s="48" t="s">
         <v>191</v>
       </c>
       <c r="B48" s="25" t="s">
@@ -8430,7 +8439,7 @@
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A49" s="50" t="s">
+      <c r="A49" s="48" t="s">
         <v>194</v>
       </c>
       <c r="B49" s="25" t="s">
@@ -8447,7 +8456,7 @@
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A50" s="50" t="s">
+      <c r="A50" s="48" t="s">
         <v>197</v>
       </c>
       <c r="B50" s="25" t="s">
@@ -8464,7 +8473,7 @@
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A51" s="50" t="s">
+      <c r="A51" s="48" t="s">
         <v>200</v>
       </c>
       <c r="B51" s="25" t="s">
@@ -8481,7 +8490,7 @@
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A52" s="50" t="s">
+      <c r="A52" s="48" t="s">
         <v>203</v>
       </c>
       <c r="B52" s="25" t="s">
@@ -8498,7 +8507,7 @@
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A53" s="50" t="s">
+      <c r="A53" s="48" t="s">
         <v>206</v>
       </c>
       <c r="B53" s="25" t="s">
@@ -8515,7 +8524,7 @@
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A54" s="50" t="s">
+      <c r="A54" s="48" t="s">
         <v>209</v>
       </c>
       <c r="B54" s="25" t="s">
@@ -8532,7 +8541,7 @@
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A55" s="50" t="s">
+      <c r="A55" s="48" t="s">
         <v>213</v>
       </c>
       <c r="B55" s="25" t="s">
@@ -8549,7 +8558,7 @@
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A56" s="50" t="s">
+      <c r="A56" s="48" t="s">
         <v>215</v>
       </c>
       <c r="B56" s="25" t="s">
@@ -8566,7 +8575,7 @@
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A57" s="50" t="s">
+      <c r="A57" s="48" t="s">
         <v>218</v>
       </c>
       <c r="B57" s="25" t="s">
@@ -8583,7 +8592,7 @@
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A58" s="50" t="s">
+      <c r="A58" s="48" t="s">
         <v>221</v>
       </c>
       <c r="B58" s="25" t="s">
@@ -8600,7 +8609,7 @@
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A59" s="51" t="s">
+      <c r="A59" s="49" t="s">
         <v>224</v>
       </c>
       <c r="B59" s="26" t="s">
@@ -8617,7 +8626,7 @@
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A60" s="51" t="s">
+      <c r="A60" s="49" t="s">
         <v>228</v>
       </c>
       <c r="B60" s="26" t="s">
@@ -8634,7 +8643,7 @@
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A61" s="51" t="s">
+      <c r="A61" s="49" t="s">
         <v>231</v>
       </c>
       <c r="B61" s="26" t="s">
@@ -8651,7 +8660,7 @@
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A62" s="51" t="s">
+      <c r="A62" s="49" t="s">
         <v>234</v>
       </c>
       <c r="B62" s="26" t="s">
@@ -8668,7 +8677,7 @@
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A63" s="51" t="s">
+      <c r="A63" s="49" t="s">
         <v>237</v>
       </c>
       <c r="B63" s="26" t="s">
@@ -8685,7 +8694,7 @@
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A64" s="51" t="s">
+      <c r="A64" s="49" t="s">
         <v>240</v>
       </c>
       <c r="B64" s="26" t="s">
@@ -8702,7 +8711,7 @@
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A65" s="51" t="s">
+      <c r="A65" s="49" t="s">
         <v>243</v>
       </c>
       <c r="B65" s="26" t="s">
@@ -8719,7 +8728,7 @@
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A66" s="51" t="s">
+      <c r="A66" s="49" t="s">
         <v>246</v>
       </c>
       <c r="B66" s="26" t="s">
@@ -8736,7 +8745,7 @@
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A67" s="51" t="s">
+      <c r="A67" s="49" t="s">
         <v>249</v>
       </c>
       <c r="B67" s="26" t="s">
@@ -8753,7 +8762,7 @@
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A68" s="51" t="s">
+      <c r="A68" s="49" t="s">
         <v>252</v>
       </c>
       <c r="B68" s="26" t="s">
@@ -8770,7 +8779,7 @@
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A69" s="51" t="s">
+      <c r="A69" s="49" t="s">
         <v>255</v>
       </c>
       <c r="B69" s="26" t="s">
@@ -8787,7 +8796,7 @@
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A70" s="51" t="s">
+      <c r="A70" s="49" t="s">
         <v>258</v>
       </c>
       <c r="B70" s="26" t="s">
@@ -8804,7 +8813,7 @@
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A71" s="51" t="s">
+      <c r="A71" s="49" t="s">
         <v>261</v>
       </c>
       <c r="B71" s="26" t="s">
@@ -8821,7 +8830,7 @@
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A72" s="51" t="s">
+      <c r="A72" s="49" t="s">
         <v>264</v>
       </c>
       <c r="B72" s="26" t="s">
@@ -8838,7 +8847,7 @@
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A73" s="51" t="s">
+      <c r="A73" s="49" t="s">
         <v>267</v>
       </c>
       <c r="B73" s="26" t="s">
@@ -8855,7 +8864,7 @@
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A74" s="51" t="s">
+      <c r="A74" s="49" t="s">
         <v>270</v>
       </c>
       <c r="B74" s="26" t="s">
@@ -8872,7 +8881,7 @@
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A75" s="51" t="s">
+      <c r="A75" s="49" t="s">
         <v>273</v>
       </c>
       <c r="B75" s="26" t="s">
@@ -8889,7 +8898,7 @@
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A76" s="51" t="s">
+      <c r="A76" s="49" t="s">
         <v>276</v>
       </c>
       <c r="B76" s="26" t="s">
@@ -8906,7 +8915,7 @@
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A77" s="51" t="s">
+      <c r="A77" s="49" t="s">
         <v>279</v>
       </c>
       <c r="B77" s="26" t="s">
@@ -8923,7 +8932,7 @@
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A78" s="51" t="s">
+      <c r="A78" s="49" t="s">
         <v>282</v>
       </c>
       <c r="B78" s="26" t="s">
@@ -8940,7 +8949,7 @@
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A79" s="51" t="s">
+      <c r="A79" s="49" t="s">
         <v>285</v>
       </c>
       <c r="B79" s="26" t="s">
@@ -8957,7 +8966,7 @@
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A80" s="51" t="s">
+      <c r="A80" s="49" t="s">
         <v>288</v>
       </c>
       <c r="B80" s="26" t="s">
@@ -8974,7 +8983,7 @@
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A81" s="51" t="s">
+      <c r="A81" s="49" t="s">
         <v>291</v>
       </c>
       <c r="B81" s="26" t="s">
@@ -8991,7 +9000,7 @@
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A82" s="51" t="s">
+      <c r="A82" s="49" t="s">
         <v>294</v>
       </c>
       <c r="B82" s="26" t="s">
@@ -9008,7 +9017,7 @@
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A83" s="51" t="s">
+      <c r="A83" s="49" t="s">
         <v>297</v>
       </c>
       <c r="B83" s="26" t="s">
@@ -9025,7 +9034,7 @@
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A84" s="51" t="s">
+      <c r="A84" s="49" t="s">
         <v>300</v>
       </c>
       <c r="B84" s="26" t="s">
@@ -9042,7 +9051,7 @@
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A85" s="51" t="s">
+      <c r="A85" s="49" t="s">
         <v>303</v>
       </c>
       <c r="B85" s="26" t="s">
@@ -9059,7 +9068,7 @@
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A86" s="51" t="s">
+      <c r="A86" s="49" t="s">
         <v>306</v>
       </c>
       <c r="B86" s="26" t="s">
@@ -9076,7 +9085,7 @@
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A87" s="51" t="s">
+      <c r="A87" s="49" t="s">
         <v>309</v>
       </c>
       <c r="B87" s="26" t="s">
@@ -9093,7 +9102,7 @@
       </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A88" s="51" t="s">
+      <c r="A88" s="49" t="s">
         <v>312</v>
       </c>
       <c r="B88" s="26" t="s">
@@ -9110,7 +9119,7 @@
       </c>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A89" s="51" t="s">
+      <c r="A89" s="49" t="s">
         <v>315</v>
       </c>
       <c r="B89" s="26" t="s">
@@ -9127,7 +9136,7 @@
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A90" s="51" t="s">
+      <c r="A90" s="49" t="s">
         <v>318</v>
       </c>
       <c r="B90" s="26" t="s">
@@ -9144,7 +9153,7 @@
       </c>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A91" s="51" t="s">
+      <c r="A91" s="49" t="s">
         <v>321</v>
       </c>
       <c r="B91" s="26" t="s">
@@ -9161,7 +9170,7 @@
       </c>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A92" s="51" t="s">
+      <c r="A92" s="49" t="s">
         <v>324</v>
       </c>
       <c r="B92" s="26" t="s">
@@ -9178,7 +9187,7 @@
       </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A93" s="51" t="s">
+      <c r="A93" s="49" t="s">
         <v>327</v>
       </c>
       <c r="B93" s="26" t="s">
@@ -9195,7 +9204,7 @@
       </c>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A94" s="51" t="s">
+      <c r="A94" s="49" t="s">
         <v>330</v>
       </c>
       <c r="B94" s="26" t="s">
@@ -9212,7 +9221,7 @@
       </c>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A95" s="51" t="s">
+      <c r="A95" s="49" t="s">
         <v>333</v>
       </c>
       <c r="B95" s="26" t="s">
@@ -9229,7 +9238,7 @@
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A96" s="51" t="s">
+      <c r="A96" s="49" t="s">
         <v>336</v>
       </c>
       <c r="B96" s="26" t="s">
@@ -9246,7 +9255,7 @@
       </c>
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A97" s="51" t="s">
+      <c r="A97" s="49" t="s">
         <v>339</v>
       </c>
       <c r="B97" s="26" t="s">
@@ -9263,7 +9272,7 @@
       </c>
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A98" s="51" t="s">
+      <c r="A98" s="49" t="s">
         <v>342</v>
       </c>
       <c r="B98" s="26" t="s">
@@ -9280,7 +9289,7 @@
       </c>
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A99" s="51" t="s">
+      <c r="A99" s="49" t="s">
         <v>345</v>
       </c>
       <c r="B99" s="26" t="s">
@@ -9297,7 +9306,7 @@
       </c>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A100" s="51" t="s">
+      <c r="A100" s="49" t="s">
         <v>348</v>
       </c>
       <c r="B100" s="26" t="s">
@@ -9314,7 +9323,7 @@
       </c>
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A101" s="51" t="s">
+      <c r="A101" s="49" t="s">
         <v>351</v>
       </c>
       <c r="B101" s="26" t="s">
@@ -9331,7 +9340,7 @@
       </c>
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A102" s="51" t="s">
+      <c r="A102" s="49" t="s">
         <v>354</v>
       </c>
       <c r="B102" s="26" t="s">
@@ -9348,7 +9357,7 @@
       </c>
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A103" s="51" t="s">
+      <c r="A103" s="49" t="s">
         <v>357</v>
       </c>
       <c r="B103" s="26" t="s">
@@ -9365,7 +9374,7 @@
       </c>
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A104" s="51" t="s">
+      <c r="A104" s="49" t="s">
         <v>360</v>
       </c>
       <c r="B104" s="26" t="s">
@@ -9382,7 +9391,7 @@
       </c>
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A105" s="51" t="s">
+      <c r="A105" s="49" t="s">
         <v>363</v>
       </c>
       <c r="B105" s="26" t="s">
@@ -9399,7 +9408,7 @@
       </c>
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A106" s="51" t="s">
+      <c r="A106" s="49" t="s">
         <v>366</v>
       </c>
       <c r="B106" s="26" t="s">
@@ -9416,7 +9425,7 @@
       </c>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A107" s="51" t="s">
+      <c r="A107" s="49" t="s">
         <v>369</v>
       </c>
       <c r="B107" s="26" t="s">
@@ -9433,7 +9442,7 @@
       </c>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A108" s="51" t="s">
+      <c r="A108" s="49" t="s">
         <v>372</v>
       </c>
       <c r="B108" s="26" t="s">
@@ -9450,7 +9459,7 @@
       </c>
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A109" s="51" t="s">
+      <c r="A109" s="49" t="s">
         <v>375</v>
       </c>
       <c r="B109" s="26" t="s">
@@ -9467,7 +9476,7 @@
       </c>
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A110" s="51" t="s">
+      <c r="A110" s="49" t="s">
         <v>379</v>
       </c>
       <c r="B110" s="26" t="s">
@@ -9484,7 +9493,7 @@
       </c>
     </row>
     <row r="111" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A111" s="51" t="s">
+      <c r="A111" s="49" t="s">
         <v>382</v>
       </c>
       <c r="B111" s="26" t="s">
@@ -9501,7 +9510,7 @@
       </c>
     </row>
     <row r="112" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A112" s="43" t="s">
+      <c r="A112" s="41" t="s">
         <v>385</v>
       </c>
       <c r="B112" s="12" t="s">
@@ -9518,7 +9527,7 @@
       </c>
     </row>
     <row r="113" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A113" s="43" t="s">
+      <c r="A113" s="41" t="s">
         <v>389</v>
       </c>
       <c r="B113" s="12" t="s">
@@ -9535,7 +9544,7 @@
       </c>
     </row>
     <row r="114" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A114" s="43" t="s">
+      <c r="A114" s="41" t="s">
         <v>392</v>
       </c>
       <c r="B114" s="12" t="s">
@@ -9552,7 +9561,7 @@
       </c>
     </row>
     <row r="115" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A115" s="43" t="s">
+      <c r="A115" s="41" t="s">
         <v>395</v>
       </c>
       <c r="B115" s="12" t="s">
@@ -9569,7 +9578,7 @@
       </c>
     </row>
     <row r="116" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A116" s="45" t="s">
+      <c r="A116" s="43" t="s">
         <v>398</v>
       </c>
       <c r="B116" s="16" t="s">
@@ -9586,7 +9595,7 @@
       </c>
     </row>
     <row r="117" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A117" s="52" t="s">
+      <c r="A117" s="50" t="s">
         <v>402</v>
       </c>
       <c r="B117" s="27" t="s">
@@ -9603,7 +9612,7 @@
       </c>
     </row>
     <row r="118" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A118" s="43" t="s">
+      <c r="A118" s="41" t="s">
         <v>406</v>
       </c>
       <c r="B118" s="12" t="s">
@@ -9620,7 +9629,7 @@
       </c>
     </row>
     <row r="119" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A119" s="43" t="s">
+      <c r="A119" s="41" t="s">
         <v>409</v>
       </c>
       <c r="B119" s="12" t="s">
@@ -9637,7 +9646,7 @@
       </c>
     </row>
     <row r="120" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A120" s="52" t="s">
+      <c r="A120" s="50" t="s">
         <v>412</v>
       </c>
       <c r="B120" s="27" t="s">
@@ -9654,7 +9663,7 @@
       </c>
     </row>
     <row r="121" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A121" s="44" t="s">
+      <c r="A121" s="42" t="s">
         <v>414</v>
       </c>
       <c r="B121" s="14" t="s">
@@ -9670,8 +9679,8 @@
         <v>417</v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A122" s="44" t="s">
+    <row r="122" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A122" s="42" t="s">
         <v>418</v>
       </c>
       <c r="B122" s="14" t="s">
@@ -9688,7 +9697,7 @@
       </c>
     </row>
     <row r="123" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A123" s="44" t="s">
+      <c r="A123" s="42" t="s">
         <v>421</v>
       </c>
       <c r="B123" s="14" t="s">
@@ -9705,7 +9714,7 @@
       </c>
     </row>
     <row r="124" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A124" s="45" t="s">
+      <c r="A124" s="43" t="s">
         <v>424</v>
       </c>
       <c r="B124" s="16" t="s">
@@ -9722,7 +9731,7 @@
       </c>
     </row>
     <row r="125" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A125" s="45" t="s">
+      <c r="A125" s="43" t="s">
         <v>427</v>
       </c>
       <c r="B125" s="16" t="s">
@@ -9739,7 +9748,7 @@
       </c>
     </row>
     <row r="126" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A126" s="45" t="s">
+      <c r="A126" s="43" t="s">
         <v>430</v>
       </c>
       <c r="B126" s="16" t="s">
@@ -9756,7 +9765,7 @@
       </c>
     </row>
     <row r="127" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A127" s="49" t="s">
+      <c r="A127" s="47" t="s">
         <v>433</v>
       </c>
       <c r="B127" s="23" t="s">
@@ -9773,7 +9782,7 @@
       </c>
     </row>
     <row r="128" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A128" s="43" t="s">
+      <c r="A128" s="41" t="s">
         <v>437</v>
       </c>
       <c r="B128" s="12" t="s">
@@ -9790,7 +9799,7 @@
       </c>
     </row>
     <row r="129" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A129" s="43" t="s">
+      <c r="A129" s="41" t="s">
         <v>441</v>
       </c>
       <c r="B129" s="12" t="s">
@@ -9807,7 +9816,7 @@
       </c>
     </row>
     <row r="130" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A130" s="43" t="s">
+      <c r="A130" s="41" t="s">
         <v>444</v>
       </c>
       <c r="B130" s="12" t="s">
@@ -9824,7 +9833,7 @@
       </c>
     </row>
     <row r="131" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A131" s="43" t="s">
+      <c r="A131" s="41" t="s">
         <v>447</v>
       </c>
       <c r="B131" s="12" t="s">

</xml_diff>